<commit_message>
fix: retain real homepage URLs in anonymized sample
</commit_message>
<xml_diff>
--- a/examples/registry/registry_sample.xlsx
+++ b/examples/registry/registry_sample.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="가상 샘플" sheetId="1" r:id="Rb1fbbc4eb43f47b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="가상 샘플" sheetId="1" r:id="R29cb667fb6ed4cfd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -59,13 +59,16 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="6">
+  <x:cellXfs count="7">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -292,13 +295,13 @@
     <x:col min="20" max="20" width="24" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="24" hidden="0" customWidth="1"/>
     <x:col min="22" max="22" width="24" hidden="0" customWidth="1"/>
-    <x:col min="23" max="23" width="24" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="52" hidden="0" customWidth="1"/>
     <x:col min="24" max="24" width="24" hidden="0" customWidth="1"/>
     <x:col min="25" max="25" width="24" hidden="0" customWidth="1"/>
     <x:col min="26" max="26" width="24" hidden="0" customWidth="1"/>
     <x:col min="27" max="27" width="24" hidden="0" customWidth="1"/>
     <x:col min="28" max="28" width="24" hidden="0" customWidth="1"/>
-    <x:col min="29" max="29" width="24" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="52" hidden="0" customWidth="1"/>
     <x:col min="30" max="30" width="24" hidden="0" customWidth="1"/>
     <x:col min="31" max="31" width="24" hidden="0" customWidth="1"/>
     <x:col min="32" max="32" width="24" hidden="0" customWidth="1"/>
@@ -434,7 +437,7 @@
         <x:v>폐간일자</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="30" customHeight="1">
+    <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="1" t="str">
         <x:v>가상기관-샘플001</x:v>
       </x:c>
@@ -477,8 +480,8 @@
       <x:c r="T2" s="1" t="str"/>
       <x:c r="U2" s="1" t="str"/>
       <x:c r="V2" s="1" t="str"/>
-      <x:c r="W2" s="1" t="str">
-        <x:v>https://sample-001.example.invalid</x:v>
+      <x:c r="W2" s="6" t="str">
+        <x:v>www.seorakcitizennews.kr</x:v>
       </x:c>
       <x:c r="X2" s="1" t="str">
         <x:v>가상사업체001</x:v>
@@ -487,8 +490,8 @@
       <x:c r="Z2" s="1" t="str"/>
       <x:c r="AA2" s="1" t="str"/>
       <x:c r="AB2" s="1" t="str"/>
-      <x:c r="AC2" s="1" t="str">
-        <x:v>https://sample-001.example.invalid</x:v>
+      <x:c r="AC2" s="6" t="str">
+        <x:v>www.seorakcitizennews.kr</x:v>
       </x:c>
       <x:c r="AD2" s="1" t="str"/>
       <x:c r="AE2" s="1" t="str">
@@ -508,7 +511,7 @@
       <x:c r="AM2" s="1" t="str"/>
       <x:c r="AN2" s="1" t="str"/>
     </x:row>
-    <x:row r="3" ht="30" customHeight="1">
+    <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="1" t="str">
         <x:v>가상기관-샘플002</x:v>
       </x:c>
@@ -551,8 +554,8 @@
       <x:c r="T3" s="1" t="str"/>
       <x:c r="U3" s="1" t="str"/>
       <x:c r="V3" s="1" t="str"/>
-      <x:c r="W3" s="1" t="str">
-        <x:v>https://sample-002.example.invalid</x:v>
+      <x:c r="W3" s="6" t="str">
+        <x:v>www.nnkorea.co.kr</x:v>
       </x:c>
       <x:c r="X3" s="1" t="str">
         <x:v>가상사업체002</x:v>
@@ -561,8 +564,8 @@
       <x:c r="Z3" s="1" t="str"/>
       <x:c r="AA3" s="1" t="str"/>
       <x:c r="AB3" s="1" t="str"/>
-      <x:c r="AC3" s="1" t="str">
-        <x:v>https://sample-002.example.invalid</x:v>
+      <x:c r="AC3" s="6" t="str">
+        <x:v>www.nnkorea.co.kr</x:v>
       </x:c>
       <x:c r="AD3" s="1" t="str"/>
       <x:c r="AE3" s="1" t="str">
@@ -582,7 +585,7 @@
       <x:c r="AM3" s="1" t="str"/>
       <x:c r="AN3" s="1" t="str"/>
     </x:row>
-    <x:row r="4" ht="30" customHeight="1">
+    <x:row r="4" ht="42" customHeight="1">
       <x:c r="A4" s="1" t="str">
         <x:v>가상기관-샘플003</x:v>
       </x:c>
@@ -625,8 +628,8 @@
       <x:c r="T4" s="1" t="str"/>
       <x:c r="U4" s="1" t="str"/>
       <x:c r="V4" s="1" t="str"/>
-      <x:c r="W4" s="1" t="str">
-        <x:v>https://sample-003.example.invalid</x:v>
+      <x:c r="W4" s="6" t="str">
+        <x:v>https://gww.scnd.kr</x:v>
       </x:c>
       <x:c r="X4" s="1" t="str">
         <x:v>가상사업체003</x:v>
@@ -635,9 +638,7 @@
       <x:c r="Z4" s="1" t="str"/>
       <x:c r="AA4" s="1" t="str"/>
       <x:c r="AB4" s="1" t="str"/>
-      <x:c r="AC4" s="1" t="str">
-        <x:v>https://sample-003.example.invalid</x:v>
-      </x:c>
+      <x:c r="AC4" s="6"/>
       <x:c r="AD4" s="1" t="str"/>
       <x:c r="AE4" s="1" t="str">
         <x:v>가상담당자003</x:v>
@@ -656,7 +657,7 @@
       <x:c r="AM4" s="1" t="str"/>
       <x:c r="AN4" s="1" t="str"/>
     </x:row>
-    <x:row r="5" ht="30" customHeight="1">
+    <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="1" t="str">
         <x:v>가상기관-샘플004</x:v>
       </x:c>
@@ -699,8 +700,8 @@
       <x:c r="T5" s="1" t="str"/>
       <x:c r="U5" s="1" t="str"/>
       <x:c r="V5" s="1" t="str"/>
-      <x:c r="W5" s="1" t="str">
-        <x:v>https://sample-004.example.invalid</x:v>
+      <x:c r="W5" s="6" t="str">
+        <x:v>www.news-b.com</x:v>
       </x:c>
       <x:c r="X5" s="1" t="str">
         <x:v>가상사업체004</x:v>
@@ -709,8 +710,8 @@
       <x:c r="Z5" s="1" t="str"/>
       <x:c r="AA5" s="1" t="str"/>
       <x:c r="AB5" s="1" t="str"/>
-      <x:c r="AC5" s="1" t="str">
-        <x:v>https://sample-004.example.invalid</x:v>
+      <x:c r="AC5" s="6" t="str">
+        <x:v>autotribune.co.kr</x:v>
       </x:c>
       <x:c r="AD5" s="1" t="str"/>
       <x:c r="AE5" s="1" t="str">
@@ -730,7 +731,7 @@
       <x:c r="AM5" s="1" t="str"/>
       <x:c r="AN5" s="1" t="str"/>
     </x:row>
-    <x:row r="6" ht="30" customHeight="1">
+    <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="1" t="str">
         <x:v>가상기관-샘플005</x:v>
       </x:c>
@@ -773,8 +774,8 @@
       <x:c r="T6" s="1" t="str"/>
       <x:c r="U6" s="1" t="str"/>
       <x:c r="V6" s="1" t="str"/>
-      <x:c r="W6" s="1" t="str">
-        <x:v>https://sample-005.example.invalid</x:v>
+      <x:c r="W6" s="6" t="str">
+        <x:v>www.daily-b.com</x:v>
       </x:c>
       <x:c r="X6" s="1" t="str">
         <x:v>가상사업체005</x:v>
@@ -783,8 +784,8 @@
       <x:c r="Z6" s="1" t="str"/>
       <x:c r="AA6" s="1" t="str"/>
       <x:c r="AB6" s="1" t="str"/>
-      <x:c r="AC6" s="1" t="str">
-        <x:v>https://sample-005.example.invalid</x:v>
+      <x:c r="AC6" s="6" t="str">
+        <x:v>autotribune.co.kr</x:v>
       </x:c>
       <x:c r="AD6" s="1" t="str"/>
       <x:c r="AE6" s="1" t="str">
@@ -804,7 +805,7 @@
       <x:c r="AM6" s="1" t="str"/>
       <x:c r="AN6" s="1" t="str"/>
     </x:row>
-    <x:row r="7" ht="30" customHeight="1">
+    <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="1" t="str">
         <x:v>가상기관-샘플006</x:v>
       </x:c>
@@ -847,8 +848,8 @@
       <x:c r="T7" s="1" t="str"/>
       <x:c r="U7" s="1" t="str"/>
       <x:c r="V7" s="1" t="str"/>
-      <x:c r="W7" s="1" t="str">
-        <x:v>https://sample-006.example.invalid</x:v>
+      <x:c r="W7" s="6" t="str">
+        <x:v>localline.kr</x:v>
       </x:c>
       <x:c r="X7" s="1" t="str">
         <x:v>가상사업체006</x:v>
@@ -857,8 +858,8 @@
       <x:c r="Z7" s="1" t="str"/>
       <x:c r="AA7" s="1" t="str"/>
       <x:c r="AB7" s="1" t="str"/>
-      <x:c r="AC7" s="1" t="str">
-        <x:v>https://sample-006.example.invalid</x:v>
+      <x:c r="AC7" s="6" t="str">
+        <x:v>localline.kr</x:v>
       </x:c>
       <x:c r="AD7" s="1" t="str"/>
       <x:c r="AE7" s="1" t="str">
@@ -878,7 +879,7 @@
       <x:c r="AM7" s="1" t="str"/>
       <x:c r="AN7" s="1" t="str"/>
     </x:row>
-    <x:row r="8" ht="30" customHeight="1">
+    <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="1" t="str">
         <x:v>가상기관-샘플007</x:v>
       </x:c>
@@ -921,8 +922,8 @@
       <x:c r="T8" s="1" t="str"/>
       <x:c r="U8" s="1" t="str"/>
       <x:c r="V8" s="1" t="str"/>
-      <x:c r="W8" s="1" t="str">
-        <x:v>https://sample-007.example.invalid</x:v>
+      <x:c r="W8" s="6" t="str">
+        <x:v>http://yesworknews.com/</x:v>
       </x:c>
       <x:c r="X8" s="1" t="str">
         <x:v>가상사업체007</x:v>
@@ -931,9 +932,7 @@
       <x:c r="Z8" s="1" t="str"/>
       <x:c r="AA8" s="1" t="str"/>
       <x:c r="AB8" s="1" t="str"/>
-      <x:c r="AC8" s="1" t="str">
-        <x:v>https://sample-007.example.invalid</x:v>
-      </x:c>
+      <x:c r="AC8" s="6"/>
       <x:c r="AD8" s="1" t="str"/>
       <x:c r="AE8" s="1" t="str">
         <x:v>가상담당자007</x:v>
@@ -952,7 +951,7 @@
       <x:c r="AM8" s="1" t="str"/>
       <x:c r="AN8" s="1" t="str"/>
     </x:row>
-    <x:row r="9" ht="30" customHeight="1">
+    <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="1" t="str">
         <x:v>가상기관-샘플008</x:v>
       </x:c>
@@ -995,8 +994,8 @@
       <x:c r="T9" s="1" t="str"/>
       <x:c r="U9" s="1" t="str"/>
       <x:c r="V9" s="1" t="str"/>
-      <x:c r="W9" s="1" t="str">
-        <x:v>https://sample-008.example.invalid</x:v>
+      <x:c r="W9" s="6" t="str">
+        <x:v>https://chungraon.com</x:v>
       </x:c>
       <x:c r="X9" s="1" t="str">
         <x:v>가상사업체008</x:v>
@@ -1005,8 +1004,8 @@
       <x:c r="Z9" s="1" t="str"/>
       <x:c r="AA9" s="1" t="str"/>
       <x:c r="AB9" s="1" t="str"/>
-      <x:c r="AC9" s="1" t="str">
-        <x:v>https://sample-008.example.invalid</x:v>
+      <x:c r="AC9" s="6" t="str">
+        <x:v>https://chungraon.com/</x:v>
       </x:c>
       <x:c r="AD9" s="1" t="str"/>
       <x:c r="AE9" s="1" t="str">
@@ -1026,7 +1025,7 @@
       <x:c r="AM9" s="1" t="str"/>
       <x:c r="AN9" s="1" t="str"/>
     </x:row>
-    <x:row r="10" ht="30" customHeight="1">
+    <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="1" t="str">
         <x:v>가상기관-샘플009</x:v>
       </x:c>
@@ -1069,8 +1068,8 @@
       <x:c r="T10" s="1" t="str"/>
       <x:c r="U10" s="1" t="str"/>
       <x:c r="V10" s="1" t="str"/>
-      <x:c r="W10" s="1" t="str">
-        <x:v>https://sample-009.example.invalid</x:v>
+      <x:c r="W10" s="6" t="str">
+        <x:v>http://cpmhj.or.kr</x:v>
       </x:c>
       <x:c r="X10" s="1" t="str">
         <x:v>가상사업체009</x:v>
@@ -1079,9 +1078,7 @@
       <x:c r="Z10" s="1" t="str"/>
       <x:c r="AA10" s="1" t="str"/>
       <x:c r="AB10" s="1" t="str"/>
-      <x:c r="AC10" s="1" t="str">
-        <x:v>https://sample-009.example.invalid</x:v>
-      </x:c>
+      <x:c r="AC10" s="6"/>
       <x:c r="AD10" s="1" t="str"/>
       <x:c r="AE10" s="1" t="str">
         <x:v>가상담당자009</x:v>
@@ -1100,7 +1097,7 @@
       <x:c r="AM10" s="1" t="str"/>
       <x:c r="AN10" s="1" t="str"/>
     </x:row>
-    <x:row r="11" ht="30" customHeight="1">
+    <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="1" t="str">
         <x:v>가상기관-샘플010</x:v>
       </x:c>
@@ -1143,8 +1140,8 @@
       <x:c r="T11" s="1" t="str"/>
       <x:c r="U11" s="1" t="str"/>
       <x:c r="V11" s="1" t="str"/>
-      <x:c r="W11" s="1" t="str">
-        <x:v>https://sample-010.example.invalid</x:v>
+      <x:c r="W11" s="6" t="str">
+        <x:v>https://hoengseongtv.kr</x:v>
       </x:c>
       <x:c r="X11" s="1" t="str">
         <x:v>가상사업체010</x:v>
@@ -1153,8 +1150,8 @@
       <x:c r="Z11" s="1" t="str"/>
       <x:c r="AA11" s="1" t="str"/>
       <x:c r="AB11" s="1" t="str"/>
-      <x:c r="AC11" s="1" t="str">
-        <x:v>https://sample-010.example.invalid</x:v>
+      <x:c r="AC11" s="6" t="str">
+        <x:v>https://hoengseongtv.kr/</x:v>
       </x:c>
       <x:c r="AD11" s="1" t="str"/>
       <x:c r="AE11" s="1" t="str">
@@ -1174,7 +1171,7 @@
       <x:c r="AM11" s="1" t="str"/>
       <x:c r="AN11" s="1" t="str"/>
     </x:row>
-    <x:row r="12" ht="30" customHeight="1">
+    <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="1" t="str">
         <x:v>가상기관-샘플011</x:v>
       </x:c>
@@ -1217,8 +1214,8 @@
       <x:c r="T12" s="1" t="str"/>
       <x:c r="U12" s="1" t="str"/>
       <x:c r="V12" s="1" t="str"/>
-      <x:c r="W12" s="1" t="str">
-        <x:v>https://sample-011.example.invalid</x:v>
+      <x:c r="W12" s="6" t="str">
+        <x:v>www.강원스마트미디어.com</x:v>
       </x:c>
       <x:c r="X12" s="1" t="str">
         <x:v>가상사업체011</x:v>
@@ -1227,9 +1224,7 @@
       <x:c r="Z12" s="1" t="str"/>
       <x:c r="AA12" s="1" t="str"/>
       <x:c r="AB12" s="1" t="str"/>
-      <x:c r="AC12" s="1" t="str">
-        <x:v>https://sample-011.example.invalid</x:v>
-      </x:c>
+      <x:c r="AC12" s="6"/>
       <x:c r="AD12" s="1" t="str"/>
       <x:c r="AE12" s="1" t="str">
         <x:v>가상담당자011</x:v>
@@ -1248,7 +1243,7 @@
       <x:c r="AM12" s="1" t="str"/>
       <x:c r="AN12" s="1" t="str"/>
     </x:row>
-    <x:row r="13" ht="30" customHeight="1">
+    <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="1" t="str">
         <x:v>가상기관-샘플012</x:v>
       </x:c>
@@ -1291,8 +1286,8 @@
       <x:c r="T13" s="1" t="str"/>
       <x:c r="U13" s="1" t="str"/>
       <x:c r="V13" s="1" t="str"/>
-      <x:c r="W13" s="1" t="str">
-        <x:v>https://sample-012.example.invalid</x:v>
+      <x:c r="W13" s="6" t="str">
+        <x:v>www.wellnesslifenews.kr</x:v>
       </x:c>
       <x:c r="X13" s="1" t="str">
         <x:v>가상사업체012</x:v>
@@ -1301,9 +1296,7 @@
       <x:c r="Z13" s="1" t="str"/>
       <x:c r="AA13" s="1" t="str"/>
       <x:c r="AB13" s="1" t="str"/>
-      <x:c r="AC13" s="1" t="str">
-        <x:v>https://sample-012.example.invalid</x:v>
-      </x:c>
+      <x:c r="AC13" s="6"/>
       <x:c r="AD13" s="1" t="str"/>
       <x:c r="AE13" s="1" t="str">
         <x:v>가상담당자012</x:v>
@@ -1322,7 +1315,7 @@
       <x:c r="AM13" s="1" t="str"/>
       <x:c r="AN13" s="1" t="str"/>
     </x:row>
-    <x:row r="14" ht="30" customHeight="1">
+    <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="1" t="str">
         <x:v>가상기관-샘플013</x:v>
       </x:c>
@@ -1365,8 +1358,8 @@
       <x:c r="T14" s="1" t="str"/>
       <x:c r="U14" s="1" t="str"/>
       <x:c r="V14" s="1" t="str"/>
-      <x:c r="W14" s="1" t="str">
-        <x:v>https://sample-013.example.invalid</x:v>
+      <x:c r="W14" s="6" t="str">
+        <x:v>https://senioredupro.com</x:v>
       </x:c>
       <x:c r="X14" s="1" t="str">
         <x:v>가상사업체013</x:v>
@@ -1375,9 +1368,7 @@
       <x:c r="Z14" s="1" t="str"/>
       <x:c r="AA14" s="1" t="str"/>
       <x:c r="AB14" s="1" t="str"/>
-      <x:c r="AC14" s="1" t="str">
-        <x:v>https://sample-013.example.invalid</x:v>
-      </x:c>
+      <x:c r="AC14" s="6"/>
       <x:c r="AD14" s="1" t="str"/>
       <x:c r="AE14" s="1" t="str">
         <x:v>가상담당자013</x:v>
@@ -1396,7 +1387,7 @@
       <x:c r="AM14" s="1" t="str"/>
       <x:c r="AN14" s="1" t="str"/>
     </x:row>
-    <x:row r="15" ht="30" customHeight="1">
+    <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="1" t="str">
         <x:v>가상기관-샘플014</x:v>
       </x:c>
@@ -1439,8 +1430,8 @@
       <x:c r="T15" s="1" t="str"/>
       <x:c r="U15" s="1" t="str"/>
       <x:c r="V15" s="1" t="str"/>
-      <x:c r="W15" s="1" t="str">
-        <x:v>https://sample-014.example.invalid</x:v>
+      <x:c r="W15" s="6" t="str">
+        <x:v>https://n-fetimes.com/</x:v>
       </x:c>
       <x:c r="X15" s="1" t="str">
         <x:v>가상사업체014</x:v>
@@ -1449,8 +1440,8 @@
       <x:c r="Z15" s="1" t="str"/>
       <x:c r="AA15" s="1" t="str"/>
       <x:c r="AB15" s="1" t="str"/>
-      <x:c r="AC15" s="1" t="str">
-        <x:v>https://sample-014.example.invalid</x:v>
+      <x:c r="AC15" s="6" t="str">
+        <x:v>https://n-fetimes.com/</x:v>
       </x:c>
       <x:c r="AD15" s="1" t="str"/>
       <x:c r="AE15" s="1" t="str">
@@ -1470,7 +1461,7 @@
       <x:c r="AM15" s="1" t="str"/>
       <x:c r="AN15" s="1" t="str"/>
     </x:row>
-    <x:row r="16" ht="30" customHeight="1">
+    <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="1" t="str">
         <x:v>가상기관-샘플015</x:v>
       </x:c>
@@ -1513,8 +1504,8 @@
       <x:c r="T16" s="1" t="str"/>
       <x:c r="U16" s="1" t="str"/>
       <x:c r="V16" s="1" t="str"/>
-      <x:c r="W16" s="1" t="str">
-        <x:v>https://sample-015.example.invalid</x:v>
+      <x:c r="W16" s="6" t="str">
+        <x:v>https://gw.breaknews.com</x:v>
       </x:c>
       <x:c r="X16" s="1" t="str">
         <x:v>가상사업체015</x:v>
@@ -1523,9 +1514,7 @@
       <x:c r="Z16" s="1" t="str"/>
       <x:c r="AA16" s="1" t="str"/>
       <x:c r="AB16" s="1" t="str"/>
-      <x:c r="AC16" s="1" t="str">
-        <x:v>https://sample-015.example.invalid</x:v>
-      </x:c>
+      <x:c r="AC16" s="6"/>
       <x:c r="AD16" s="1" t="str"/>
       <x:c r="AE16" s="1" t="str">
         <x:v>가상담당자015</x:v>
@@ -1544,7 +1533,7 @@
       <x:c r="AM16" s="1" t="str"/>
       <x:c r="AN16" s="1" t="str"/>
     </x:row>
-    <x:row r="17" ht="30" customHeight="1">
+    <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="1" t="str">
         <x:v>가상기관-샘플016</x:v>
       </x:c>
@@ -1587,8 +1576,8 @@
       <x:c r="T17" s="1" t="str"/>
       <x:c r="U17" s="1" t="str"/>
       <x:c r="V17" s="1" t="str"/>
-      <x:c r="W17" s="1" t="str">
-        <x:v>https://sample-016.example.invalid</x:v>
+      <x:c r="W17" s="6" t="str">
+        <x:v>servicenews.co.kr</x:v>
       </x:c>
       <x:c r="X17" s="1" t="str">
         <x:v>가상사업체016</x:v>
@@ -1597,8 +1586,8 @@
       <x:c r="Z17" s="1" t="str"/>
       <x:c r="AA17" s="1" t="str"/>
       <x:c r="AB17" s="1" t="str"/>
-      <x:c r="AC17" s="1" t="str">
-        <x:v>https://sample-016.example.invalid</x:v>
+      <x:c r="AC17" s="6" t="str">
+        <x:v>servicenews.co.kr</x:v>
       </x:c>
       <x:c r="AD17" s="1" t="str"/>
       <x:c r="AE17" s="1" t="str">
@@ -1618,7 +1607,7 @@
       <x:c r="AM17" s="1" t="str"/>
       <x:c r="AN17" s="1" t="str"/>
     </x:row>
-    <x:row r="18" ht="30" customHeight="1">
+    <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="1" t="str">
         <x:v>가상기관-샘플017</x:v>
       </x:c>
@@ -1661,8 +1650,8 @@
       <x:c r="T18" s="1" t="str"/>
       <x:c r="U18" s="1" t="str"/>
       <x:c r="V18" s="1" t="str"/>
-      <x:c r="W18" s="1" t="str">
-        <x:v>https://sample-017.example.invalid</x:v>
+      <x:c r="W18" s="6" t="str">
+        <x:v>www.smartagrinews.com</x:v>
       </x:c>
       <x:c r="X18" s="1" t="str">
         <x:v>가상사업체017</x:v>
@@ -1671,9 +1660,7 @@
       <x:c r="Z18" s="1" t="str"/>
       <x:c r="AA18" s="1" t="str"/>
       <x:c r="AB18" s="1" t="str"/>
-      <x:c r="AC18" s="1" t="str">
-        <x:v>https://sample-017.example.invalid</x:v>
-      </x:c>
+      <x:c r="AC18" s="6"/>
       <x:c r="AD18" s="1" t="str"/>
       <x:c r="AE18" s="1" t="str">
         <x:v>가상담당자017</x:v>
@@ -1692,7 +1679,7 @@
       <x:c r="AM18" s="1" t="str"/>
       <x:c r="AN18" s="1" t="str"/>
     </x:row>
-    <x:row r="19" ht="30" customHeight="1">
+    <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="1" t="str">
         <x:v>가상기관-샘플018</x:v>
       </x:c>
@@ -1735,8 +1722,8 @@
       <x:c r="T19" s="1" t="str"/>
       <x:c r="U19" s="1" t="str"/>
       <x:c r="V19" s="1" t="str"/>
-      <x:c r="W19" s="1" t="str">
-        <x:v>https://sample-018.example.invalid</x:v>
+      <x:c r="W19" s="6" t="str">
+        <x:v>www.headline21.com</x:v>
       </x:c>
       <x:c r="X19" s="1" t="str">
         <x:v>가상사업체018</x:v>
@@ -1745,9 +1732,7 @@
       <x:c r="Z19" s="1" t="str"/>
       <x:c r="AA19" s="1" t="str"/>
       <x:c r="AB19" s="1" t="str"/>
-      <x:c r="AC19" s="1" t="str">
-        <x:v>https://sample-018.example.invalid</x:v>
-      </x:c>
+      <x:c r="AC19" s="6"/>
       <x:c r="AD19" s="1" t="str"/>
       <x:c r="AE19" s="1" t="str">
         <x:v>가상담당자018</x:v>
@@ -1766,7 +1751,7 @@
       <x:c r="AM19" s="1" t="str"/>
       <x:c r="AN19" s="1" t="str"/>
     </x:row>
-    <x:row r="20" ht="30" customHeight="1">
+    <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="1" t="str">
         <x:v>가상기관-샘플019</x:v>
       </x:c>
@@ -1809,8 +1794,8 @@
       <x:c r="T20" s="1" t="str"/>
       <x:c r="U20" s="1" t="str"/>
       <x:c r="V20" s="1" t="str"/>
-      <x:c r="W20" s="1" t="str">
-        <x:v>https://sample-019.example.invalid</x:v>
+      <x:c r="W20" s="6" t="str">
+        <x:v>hctoday.kr</x:v>
       </x:c>
       <x:c r="X20" s="1" t="str">
         <x:v>가상사업체019</x:v>
@@ -1819,9 +1804,7 @@
       <x:c r="Z20" s="1" t="str"/>
       <x:c r="AA20" s="1" t="str"/>
       <x:c r="AB20" s="1" t="str"/>
-      <x:c r="AC20" s="1" t="str">
-        <x:v>https://sample-019.example.invalid</x:v>
-      </x:c>
+      <x:c r="AC20" s="6"/>
       <x:c r="AD20" s="1" t="str"/>
       <x:c r="AE20" s="1" t="str">
         <x:v>가상담당자019</x:v>
@@ -1840,7 +1823,7 @@
       <x:c r="AM20" s="1" t="str"/>
       <x:c r="AN20" s="1" t="str"/>
     </x:row>
-    <x:row r="21" ht="30" customHeight="1">
+    <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="1" t="str">
         <x:v>가상기관-샘플020</x:v>
       </x:c>
@@ -1883,8 +1866,8 @@
       <x:c r="T21" s="1" t="str"/>
       <x:c r="U21" s="1" t="str"/>
       <x:c r="V21" s="1" t="str"/>
-      <x:c r="W21" s="1" t="str">
-        <x:v>https://sample-020.example.invalid</x:v>
+      <x:c r="W21" s="6" t="str">
+        <x:v>인제투데이.com</x:v>
       </x:c>
       <x:c r="X21" s="1" t="str">
         <x:v>가상사업체020</x:v>
@@ -1893,9 +1876,7 @@
       <x:c r="Z21" s="1" t="str"/>
       <x:c r="AA21" s="1" t="str"/>
       <x:c r="AB21" s="1" t="str"/>
-      <x:c r="AC21" s="1" t="str">
-        <x:v>https://sample-020.example.invalid</x:v>
-      </x:c>
+      <x:c r="AC21" s="6"/>
       <x:c r="AD21" s="1" t="str"/>
       <x:c r="AE21" s="1" t="str">
         <x:v>가상담당자020</x:v>

</xml_diff>